<commit_message>
Link pricing table prices to the original budget sheet via formulas
السعر column now pulls live from "الميزانية الأصلية" cells instead of
hardcoded numbers (row 1 stays a manual input since it's a given
value with no clean source breakdown). Added a small assumptions
block with editable weight cells for the estimated 3-way split, and
converted the original-budget sheet's own subtotals to SUM formulas
so the whole workbook recalculates from the raw line items.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YCs2bzKSRgNMCsEjeM1Z1F
</commit_message>
<xml_diff>
--- a/output/Pricing_Table.xlsx
+++ b/output/Pricing_Table.xlsx
@@ -21,8 +21,38 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="F2" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="FreeSans"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">قيمة معطاة مسبقًا من العميل لبند منطقة الصانع الصغير — إدخال يدوي، غير مشتقة من شيت الميزانية الأصلية</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="85">
   <si>
     <t xml:space="preserve">م</t>
   </si>
@@ -117,7 +147,22 @@
     <t xml:space="preserve">الإجمالي شامل الضريبة</t>
   </si>
   <si>
-    <t xml:space="preserve">ملاحظة: البنود 2، 5، 6، 8، 9 موزّعة بالتوزيع التقديري لعدم وجود تطابق مباشر بالاسم مع بنود الميزانية الأصلية — راجع شيت "مصدر الأرقام" للتفاصيل.</t>
+    <t xml:space="preserve">افتراضات التوزيع التقديري (بند 2 + بند 5 + بند 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إجمالي حصة (سعودي بيوتي + مسرح الصناعة + نقاط الضيافة) = (الصانع الصغير الكامل ناقص القيمة المعطاة للبند 1) + معدات وتطوير محتوى "تجارب متنوعة" (بدون تصميم الفكرة ومرحلة التشغيل، المخصصين للبندين 8 و9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وزن منطقة سعودي بيوتي (بند 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وزن مسرح الصناعة (بند 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وزن نقاط الضيافة السعودية (بند 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عدّل نسب الأوزان الصفراء أعلاه حسب الحاجة — بنود 2، 5، 6 ستُعاد حسابها تلقائيًا. تغيير أي رقم في شيت "الميزانية الأصلية" ينعكس تلقائيًا على كل أسعار هذا الجدول (ما عدا بند 1 المعطى مسبقًا).</t>
   </si>
   <si>
     <t xml:space="preserve">التفاصيل</t>
@@ -259,17 +304,21 @@
   </si>
   <si>
     <t xml:space="preserve">ملاحظة ختامية: البنود 2، 5، 6، 8، 9 تتضمن افتراضات توزيع تقديرية (موضحة أعلاه) نظرًا لعدم وجود تطابق مباشر بالاسم بين بنود الميزانية الأصلية وبنود جدول التسعير — يُنصح بمراجعتها مع صاحب المشروع.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ملاحظة تقنية: كل الأسعار في شيت "جدول التسعير" (ما عدا البند 1) أصبحت صيغ مرتبطة مباشرة بخلايا شيت "الميزانية الأصلية" — أي تعديل على أرقام الميزانية الأصلية أو على نسب التوزيع الصفراء (صف 18-20 في جدول التسعير) ينعكس تلقائيًا على الأسعار والإجمالي.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,8 +356,38 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -322,6 +401,16 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="FreeSans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
@@ -329,8 +418,17 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F4E78"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -353,6 +451,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
         <bgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -405,11 +509,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -426,47 +534,79 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -722,292 +862,365 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="6" t="n">
         <v>5985779</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="5" t="n">
-        <v>1018184.59</v>
+      <c r="F3" s="7" t="n">
+        <f aca="false">$F$17*$F$18</f>
+        <v>1018184.3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!C21+'الميزانية الأصلية'!C22+'الميزانية الأصلية'!C23</f>
         <v>5283787</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!C17</f>
         <v>580880</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>1163639.54</v>
+      <c r="F6" s="7" t="n">
+        <f aca="false">$F$17*$F$19</f>
+        <v>1163639.2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>727274.71</v>
+      <c r="F7" s="7" t="n">
+        <f aca="false">$F$17*$F$20</f>
+        <v>727274.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>1050</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!D2+'الميزانية الأصلية'!D32</f>
         <v>13200000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!C16+'الميزانية الأصلية'!C20+'الميزانية الأصلية'!C26</f>
         <v>142036.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!C18+'الميزانية الأصلية'!C24+'الميزانية الأصلية'!C30+'الميزانية الأصلية'!D33</f>
         <v>1644842.66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="7" t="n">
+        <f aca="false">'الميزانية الأصلية'!D6</f>
         <v>7000000</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7" t="n">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="n">
         <f aca="false">SUM(F2:F11)</f>
-        <v>36746424</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+        <v>36746423.16</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7" t="n">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9" t="n">
         <f aca="false">F12*0.15</f>
-        <v>5511963.6</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
+        <v>5511963.474</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="9" t="n">
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="11" t="n">
         <f aca="false">F12+F13</f>
-        <v>42258387.6</v>
+        <v>42258386.634</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="15" t="n">
+        <f aca="false">SUM('الميزانية الأصلية'!C9:C14)-F2+SUM('الميزانية الأصلية'!C27:C29)</f>
+        <v>2909098</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="16" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="16" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="16" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1016,6 +1229,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1027,367 +1241,372 @@
   <dimension ref="A1:D37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="7" t="n">
+      <c r="B1" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="9" t="n">
         <v>10500000</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="5" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="21" t="n">
         <v>4500000</v>
       </c>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3" t="s">
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="12"/>
-      <c r="D6" s="7" t="n">
+      <c r="C6" s="19"/>
+      <c r="D6" s="9" t="n">
+        <f aca="false">SUM(C4:C5)</f>
         <v>7000000</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="5" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="21" t="n">
         <v>95859</v>
       </c>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="5" t="n">
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="21" t="n">
         <v>2325475</v>
       </c>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="5" t="n">
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="21" t="n">
         <v>1175430</v>
       </c>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="5" t="n">
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="21" t="n">
         <v>64445</v>
       </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="5" t="n">
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="21" t="n">
         <v>830016</v>
       </c>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3" t="s">
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20"/>
+      <c r="B15" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C16" s="21" t="n">
+        <v>24833</v>
+      </c>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>580880</v>
+      </c>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>522602.66</v>
+      </c>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>79460</v>
+      </c>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="21" t="n">
         <v>3500000</v>
       </c>
-      <c r="D14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13" t="s">
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>1578972</v>
+      </c>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="21" t="n">
+        <v>204815</v>
+      </c>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>461120</v>
+      </c>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="21" t="n">
+        <v>37743.5</v>
+      </c>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>24833</v>
-      </c>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>580880</v>
-      </c>
-      <c r="D17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>522602.66</v>
-      </c>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13" t="s">
+      <c r="C27" s="21" t="n">
+        <v>441825</v>
+      </c>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>79460</v>
-      </c>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="D21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>1578972</v>
-      </c>
-      <c r="D22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3" t="s">
+      <c r="C28" s="21" t="n">
+        <v>193992</v>
+      </c>
+      <c r="D28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="5" t="n">
-        <v>204815</v>
-      </c>
-      <c r="D23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="5" t="n">
+      <c r="C29" s="21" t="n">
+        <v>267835</v>
+      </c>
+      <c r="D29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="21" t="n">
         <v>461120</v>
       </c>
-      <c r="D24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>37743.5</v>
-      </c>
-      <c r="D26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>441825</v>
-      </c>
-      <c r="D27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>193992</v>
-      </c>
-      <c r="D28" s="3"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>267835</v>
-      </c>
-      <c r="D29" s="3"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>461120</v>
-      </c>
-      <c r="D30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12" t="s">
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19"/>
+      <c r="B31" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="9" t="n">
+        <f aca="false">SUM(C9:C30)</f>
+        <v>16346423.16</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" s="19"/>
+      <c r="D32" s="9" t="n">
+        <v>2700000</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="7" t="n">
-        <v>16346424</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="7" t="n">
-        <v>2700000</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="12"/>
-      <c r="D33" s="7" t="n">
+      <c r="B33" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="9" t="n">
         <v>200000</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="7" t="n">
-        <v>36746424</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="7" t="n">
-        <v>5511964</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="7" t="n">
-        <v>42258387</v>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="9" t="n">
+        <f aca="false">D2+D6+D31+D32+D33</f>
+        <v>36746423.16</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="9" t="n">
+        <f aca="false">D35*0.15</f>
+        <v>5511963.474</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="9" t="n">
+        <f aca="false">D35+D36</f>
+        <v>42258386.634</v>
       </c>
     </row>
   </sheetData>
@@ -1406,102 +1625,109 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="100"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>59</v>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>61</v>
+      <c r="A2" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>63</v>
+      <c r="A3" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>65</v>
+      <c r="A4" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>67</v>
+      <c r="A5" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>69</v>
+      <c r="A6" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>71</v>
+      <c r="A7" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>73</v>
+      <c r="A8" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>75</v>
+      <c r="A9" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>77</v>
+      <c r="A10" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="15"/>
+      <c r="A12" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="23"/>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A14:B14"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>